<commit_message>
Système de gestion de stock automatisé : 4 workflows (vente, arrivage, point du matin, bilan), template avec Arrivages et quantité à commander, PDF explicatif
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RavxZb3XR9FuiiE8cVSRNP
</commit_message>
<xml_diff>
--- a/produits/templates-entreprises/gestion_de_stock.xlsx
+++ b/produits/templates-entreprises/gestion_de_stock.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="78">
   <si>
     <t xml:space="preserve">Gestion de stock : mode d'emploi</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t xml:space="preserve">4. Le seuil d'alerte : en dessous de cette quantité, le produit passe en « À commander ».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Facultatif : le fournisseur et son téléphone. La colonne « Quantité à commander » propose de quoi remonter le stock au double du seuil d'alerte.</t>
   </si>
   <si>
     <t xml:space="preserve">Étape 2 : chaque jour (onglet Mouvements)</t>
@@ -178,6 +181,15 @@
     <t xml:space="preserve">État</t>
   </si>
   <si>
+    <t xml:space="preserve">Fournisseur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tél. fournisseur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantité à commander</t>
+  </si>
+  <si>
     <t xml:space="preserve">P001</t>
   </si>
   <si>
@@ -190,6 +202,9 @@
     <t xml:space="preserve">sac</t>
   </si>
   <si>
+    <t xml:space="preserve">EXEMPLE - Grossiste A</t>
+  </si>
+  <si>
     <t xml:space="preserve">P002</t>
   </si>
   <si>
@@ -197,6 +212,9 @@
   </si>
   <si>
     <t xml:space="preserve">bidon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXEMPLE - Grossiste B</t>
   </si>
   <si>
     <t xml:space="preserve">Mouvements de stock</t>
@@ -865,7 +883,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:B28"/>
+  <dimension ref="B1:B29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -927,47 +945,47 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="2" t="s">
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="3" t="s">
+    <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="2" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="3" t="s">
+    <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="2" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="3" t="s">
+    <row r="25" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="3" t="s">
         <v>19</v>
       </c>
@@ -975,6 +993,11 @@
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="3" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="3" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1004,40 +1027,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C4" s="9" t="n">
         <f aca="true">TODAY()</f>
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C7" s="12" t="n">
         <f aca="false">COUNTA(Produits!$A$5:$A$204)</f>
@@ -1056,31 +1079,31 @@
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C9" s="12" t="n">
         <f aca="false">COUNTIF(Produits!$M$5:$M$204,"À commander")</f>
         <v>1</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C10" s="12" t="n">
         <f aca="false">COUNTIF(Produits!$M$5:$M$204,"Rupture")</f>
         <v>0</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1123,12 +1146,12 @@
         <v>45</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C16" s="15" t="n">
         <f aca="false">IF(C12=0,"-",C15/C12)</f>
@@ -1161,7 +1184,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M204"/>
+  <dimension ref="A1:P204"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -1174,71 +1197,83 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J4" s="18" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M4" s="18" t="s">
-        <v>50</v>
+        <v>51</v>
+      </c>
+      <c r="N4" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="O4" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="P4" s="18" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E5" s="20" t="n">
         <v>30</v>
@@ -1272,19 +1307,27 @@
         <f aca="false">IF($A5="","",IF($K5&lt;=0,"Rupture",IF($K5&lt;=N($H5),"À commander","OK")))</f>
         <v>OK</v>
       </c>
+      <c r="N5" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="O5" s="23"/>
+      <c r="P5" s="21" t="n">
+        <f aca="false">IF($A5="","",IF($K5&lt;=N($H5),MAX(0,2*N($H5)-$K5),0))</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E6" s="20" t="n">
         <v>12</v>
@@ -1317,6 +1360,14 @@
       <c r="M6" s="22" t="str">
         <f aca="false">IF($A6="","",IF($K6&lt;=0,"Rupture",IF($K6&lt;=N($H6),"À commander","OK")))</f>
         <v>À commander</v>
+      </c>
+      <c r="N6" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="O6" s="23"/>
+      <c r="P6" s="21" t="n">
+        <f aca="false">IF($A6="","",IF($K6&lt;=N($H6),MAX(0,2*N($H6)-$K6),0))</f>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1348,6 +1399,12 @@
         <f aca="false">IF($A7="","",IF($K7&lt;=0,"Rupture",IF($K7&lt;=N($H7),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N7" s="23"/>
+      <c r="O7" s="23"/>
+      <c r="P7" s="21" t="str">
+        <f aca="false">IF($A7="","",IF($K7&lt;=N($H7),MAX(0,2*N($H7)-$K7),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23"/>
@@ -1378,6 +1435,12 @@
         <f aca="false">IF($A8="","",IF($K8&lt;=0,"Rupture",IF($K8&lt;=N($H8),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N8" s="23"/>
+      <c r="O8" s="23"/>
+      <c r="P8" s="21" t="str">
+        <f aca="false">IF($A8="","",IF($K8&lt;=N($H8),MAX(0,2*N($H8)-$K8),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23"/>
@@ -1408,6 +1471,12 @@
         <f aca="false">IF($A9="","",IF($K9&lt;=0,"Rupture",IF($K9&lt;=N($H9),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N9" s="23"/>
+      <c r="O9" s="23"/>
+      <c r="P9" s="21" t="str">
+        <f aca="false">IF($A9="","",IF($K9&lt;=N($H9),MAX(0,2*N($H9)-$K9),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="23"/>
@@ -1438,6 +1507,12 @@
         <f aca="false">IF($A10="","",IF($K10&lt;=0,"Rupture",IF($K10&lt;=N($H10),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N10" s="23"/>
+      <c r="O10" s="23"/>
+      <c r="P10" s="21" t="str">
+        <f aca="false">IF($A10="","",IF($K10&lt;=N($H10),MAX(0,2*N($H10)-$K10),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23"/>
@@ -1468,6 +1543,12 @@
         <f aca="false">IF($A11="","",IF($K11&lt;=0,"Rupture",IF($K11&lt;=N($H11),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N11" s="23"/>
+      <c r="O11" s="23"/>
+      <c r="P11" s="21" t="str">
+        <f aca="false">IF($A11="","",IF($K11&lt;=N($H11),MAX(0,2*N($H11)-$K11),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23"/>
@@ -1498,6 +1579,12 @@
         <f aca="false">IF($A12="","",IF($K12&lt;=0,"Rupture",IF($K12&lt;=N($H12),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N12" s="23"/>
+      <c r="O12" s="23"/>
+      <c r="P12" s="21" t="str">
+        <f aca="false">IF($A12="","",IF($K12&lt;=N($H12),MAX(0,2*N($H12)-$K12),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="23"/>
@@ -1528,6 +1615,12 @@
         <f aca="false">IF($A13="","",IF($K13&lt;=0,"Rupture",IF($K13&lt;=N($H13),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N13" s="23"/>
+      <c r="O13" s="23"/>
+      <c r="P13" s="21" t="str">
+        <f aca="false">IF($A13="","",IF($K13&lt;=N($H13),MAX(0,2*N($H13)-$K13),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23"/>
@@ -1558,6 +1651,12 @@
         <f aca="false">IF($A14="","",IF($K14&lt;=0,"Rupture",IF($K14&lt;=N($H14),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N14" s="23"/>
+      <c r="O14" s="23"/>
+      <c r="P14" s="21" t="str">
+        <f aca="false">IF($A14="","",IF($K14&lt;=N($H14),MAX(0,2*N($H14)-$K14),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="23"/>
@@ -1588,6 +1687,12 @@
         <f aca="false">IF($A15="","",IF($K15&lt;=0,"Rupture",IF($K15&lt;=N($H15),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N15" s="23"/>
+      <c r="O15" s="23"/>
+      <c r="P15" s="21" t="str">
+        <f aca="false">IF($A15="","",IF($K15&lt;=N($H15),MAX(0,2*N($H15)-$K15),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="23"/>
@@ -1618,6 +1723,12 @@
         <f aca="false">IF($A16="","",IF($K16&lt;=0,"Rupture",IF($K16&lt;=N($H16),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N16" s="23"/>
+      <c r="O16" s="23"/>
+      <c r="P16" s="21" t="str">
+        <f aca="false">IF($A16="","",IF($K16&lt;=N($H16),MAX(0,2*N($H16)-$K16),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23"/>
@@ -1648,6 +1759,12 @@
         <f aca="false">IF($A17="","",IF($K17&lt;=0,"Rupture",IF($K17&lt;=N($H17),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N17" s="23"/>
+      <c r="O17" s="23"/>
+      <c r="P17" s="21" t="str">
+        <f aca="false">IF($A17="","",IF($K17&lt;=N($H17),MAX(0,2*N($H17)-$K17),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23"/>
@@ -1678,6 +1795,12 @@
         <f aca="false">IF($A18="","",IF($K18&lt;=0,"Rupture",IF($K18&lt;=N($H18),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N18" s="23"/>
+      <c r="O18" s="23"/>
+      <c r="P18" s="21" t="str">
+        <f aca="false">IF($A18="","",IF($K18&lt;=N($H18),MAX(0,2*N($H18)-$K18),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="23"/>
@@ -1708,6 +1831,12 @@
         <f aca="false">IF($A19="","",IF($K19&lt;=0,"Rupture",IF($K19&lt;=N($H19),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N19" s="23"/>
+      <c r="O19" s="23"/>
+      <c r="P19" s="21" t="str">
+        <f aca="false">IF($A19="","",IF($K19&lt;=N($H19),MAX(0,2*N($H19)-$K19),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="23"/>
@@ -1738,6 +1867,12 @@
         <f aca="false">IF($A20="","",IF($K20&lt;=0,"Rupture",IF($K20&lt;=N($H20),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N20" s="23"/>
+      <c r="O20" s="23"/>
+      <c r="P20" s="21" t="str">
+        <f aca="false">IF($A20="","",IF($K20&lt;=N($H20),MAX(0,2*N($H20)-$K20),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="23"/>
@@ -1768,6 +1903,12 @@
         <f aca="false">IF($A21="","",IF($K21&lt;=0,"Rupture",IF($K21&lt;=N($H21),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N21" s="23"/>
+      <c r="O21" s="23"/>
+      <c r="P21" s="21" t="str">
+        <f aca="false">IF($A21="","",IF($K21&lt;=N($H21),MAX(0,2*N($H21)-$K21),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="23"/>
@@ -1798,6 +1939,12 @@
         <f aca="false">IF($A22="","",IF($K22&lt;=0,"Rupture",IF($K22&lt;=N($H22),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N22" s="23"/>
+      <c r="O22" s="23"/>
+      <c r="P22" s="21" t="str">
+        <f aca="false">IF($A22="","",IF($K22&lt;=N($H22),MAX(0,2*N($H22)-$K22),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23"/>
@@ -1828,6 +1975,12 @@
         <f aca="false">IF($A23="","",IF($K23&lt;=0,"Rupture",IF($K23&lt;=N($H23),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N23" s="23"/>
+      <c r="O23" s="23"/>
+      <c r="P23" s="21" t="str">
+        <f aca="false">IF($A23="","",IF($K23&lt;=N($H23),MAX(0,2*N($H23)-$K23),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="23"/>
@@ -1858,6 +2011,12 @@
         <f aca="false">IF($A24="","",IF($K24&lt;=0,"Rupture",IF($K24&lt;=N($H24),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N24" s="23"/>
+      <c r="O24" s="23"/>
+      <c r="P24" s="21" t="str">
+        <f aca="false">IF($A24="","",IF($K24&lt;=N($H24),MAX(0,2*N($H24)-$K24),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="23"/>
@@ -1888,6 +2047,12 @@
         <f aca="false">IF($A25="","",IF($K25&lt;=0,"Rupture",IF($K25&lt;=N($H25),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N25" s="23"/>
+      <c r="O25" s="23"/>
+      <c r="P25" s="21" t="str">
+        <f aca="false">IF($A25="","",IF($K25&lt;=N($H25),MAX(0,2*N($H25)-$K25),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="23"/>
@@ -1918,6 +2083,12 @@
         <f aca="false">IF($A26="","",IF($K26&lt;=0,"Rupture",IF($K26&lt;=N($H26),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N26" s="23"/>
+      <c r="O26" s="23"/>
+      <c r="P26" s="21" t="str">
+        <f aca="false">IF($A26="","",IF($K26&lt;=N($H26),MAX(0,2*N($H26)-$K26),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="23"/>
@@ -1948,6 +2119,12 @@
         <f aca="false">IF($A27="","",IF($K27&lt;=0,"Rupture",IF($K27&lt;=N($H27),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N27" s="23"/>
+      <c r="O27" s="23"/>
+      <c r="P27" s="21" t="str">
+        <f aca="false">IF($A27="","",IF($K27&lt;=N($H27),MAX(0,2*N($H27)-$K27),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="23"/>
@@ -1978,6 +2155,12 @@
         <f aca="false">IF($A28="","",IF($K28&lt;=0,"Rupture",IF($K28&lt;=N($H28),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N28" s="23"/>
+      <c r="O28" s="23"/>
+      <c r="P28" s="21" t="str">
+        <f aca="false">IF($A28="","",IF($K28&lt;=N($H28),MAX(0,2*N($H28)-$K28),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="23"/>
@@ -2008,6 +2191,12 @@
         <f aca="false">IF($A29="","",IF($K29&lt;=0,"Rupture",IF($K29&lt;=N($H29),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N29" s="23"/>
+      <c r="O29" s="23"/>
+      <c r="P29" s="21" t="str">
+        <f aca="false">IF($A29="","",IF($K29&lt;=N($H29),MAX(0,2*N($H29)-$K29),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="23"/>
@@ -2038,6 +2227,12 @@
         <f aca="false">IF($A30="","",IF($K30&lt;=0,"Rupture",IF($K30&lt;=N($H30),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N30" s="23"/>
+      <c r="O30" s="23"/>
+      <c r="P30" s="21" t="str">
+        <f aca="false">IF($A30="","",IF($K30&lt;=N($H30),MAX(0,2*N($H30)-$K30),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="23"/>
@@ -2068,6 +2263,12 @@
         <f aca="false">IF($A31="","",IF($K31&lt;=0,"Rupture",IF($K31&lt;=N($H31),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N31" s="23"/>
+      <c r="O31" s="23"/>
+      <c r="P31" s="21" t="str">
+        <f aca="false">IF($A31="","",IF($K31&lt;=N($H31),MAX(0,2*N($H31)-$K31),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="23"/>
@@ -2098,6 +2299,12 @@
         <f aca="false">IF($A32="","",IF($K32&lt;=0,"Rupture",IF($K32&lt;=N($H32),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N32" s="23"/>
+      <c r="O32" s="23"/>
+      <c r="P32" s="21" t="str">
+        <f aca="false">IF($A32="","",IF($K32&lt;=N($H32),MAX(0,2*N($H32)-$K32),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="23"/>
@@ -2128,6 +2335,12 @@
         <f aca="false">IF($A33="","",IF($K33&lt;=0,"Rupture",IF($K33&lt;=N($H33),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N33" s="23"/>
+      <c r="O33" s="23"/>
+      <c r="P33" s="21" t="str">
+        <f aca="false">IF($A33="","",IF($K33&lt;=N($H33),MAX(0,2*N($H33)-$K33),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="23"/>
@@ -2158,6 +2371,12 @@
         <f aca="false">IF($A34="","",IF($K34&lt;=0,"Rupture",IF($K34&lt;=N($H34),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N34" s="23"/>
+      <c r="O34" s="23"/>
+      <c r="P34" s="21" t="str">
+        <f aca="false">IF($A34="","",IF($K34&lt;=N($H34),MAX(0,2*N($H34)-$K34),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="23"/>
@@ -2188,6 +2407,12 @@
         <f aca="false">IF($A35="","",IF($K35&lt;=0,"Rupture",IF($K35&lt;=N($H35),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N35" s="23"/>
+      <c r="O35" s="23"/>
+      <c r="P35" s="21" t="str">
+        <f aca="false">IF($A35="","",IF($K35&lt;=N($H35),MAX(0,2*N($H35)-$K35),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="23"/>
@@ -2218,6 +2443,12 @@
         <f aca="false">IF($A36="","",IF($K36&lt;=0,"Rupture",IF($K36&lt;=N($H36),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N36" s="23"/>
+      <c r="O36" s="23"/>
+      <c r="P36" s="21" t="str">
+        <f aca="false">IF($A36="","",IF($K36&lt;=N($H36),MAX(0,2*N($H36)-$K36),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="23"/>
@@ -2248,6 +2479,12 @@
         <f aca="false">IF($A37="","",IF($K37&lt;=0,"Rupture",IF($K37&lt;=N($H37),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N37" s="23"/>
+      <c r="O37" s="23"/>
+      <c r="P37" s="21" t="str">
+        <f aca="false">IF($A37="","",IF($K37&lt;=N($H37),MAX(0,2*N($H37)-$K37),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="23"/>
@@ -2278,6 +2515,12 @@
         <f aca="false">IF($A38="","",IF($K38&lt;=0,"Rupture",IF($K38&lt;=N($H38),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N38" s="23"/>
+      <c r="O38" s="23"/>
+      <c r="P38" s="21" t="str">
+        <f aca="false">IF($A38="","",IF($K38&lt;=N($H38),MAX(0,2*N($H38)-$K38),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="23"/>
@@ -2308,6 +2551,12 @@
         <f aca="false">IF($A39="","",IF($K39&lt;=0,"Rupture",IF($K39&lt;=N($H39),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N39" s="23"/>
+      <c r="O39" s="23"/>
+      <c r="P39" s="21" t="str">
+        <f aca="false">IF($A39="","",IF($K39&lt;=N($H39),MAX(0,2*N($H39)-$K39),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="23"/>
@@ -2338,6 +2587,12 @@
         <f aca="false">IF($A40="","",IF($K40&lt;=0,"Rupture",IF($K40&lt;=N($H40),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N40" s="23"/>
+      <c r="O40" s="23"/>
+      <c r="P40" s="21" t="str">
+        <f aca="false">IF($A40="","",IF($K40&lt;=N($H40),MAX(0,2*N($H40)-$K40),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="23"/>
@@ -2368,6 +2623,12 @@
         <f aca="false">IF($A41="","",IF($K41&lt;=0,"Rupture",IF($K41&lt;=N($H41),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N41" s="23"/>
+      <c r="O41" s="23"/>
+      <c r="P41" s="21" t="str">
+        <f aca="false">IF($A41="","",IF($K41&lt;=N($H41),MAX(0,2*N($H41)-$K41),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="23"/>
@@ -2398,6 +2659,12 @@
         <f aca="false">IF($A42="","",IF($K42&lt;=0,"Rupture",IF($K42&lt;=N($H42),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N42" s="23"/>
+      <c r="O42" s="23"/>
+      <c r="P42" s="21" t="str">
+        <f aca="false">IF($A42="","",IF($K42&lt;=N($H42),MAX(0,2*N($H42)-$K42),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="23"/>
@@ -2428,6 +2695,12 @@
         <f aca="false">IF($A43="","",IF($K43&lt;=0,"Rupture",IF($K43&lt;=N($H43),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N43" s="23"/>
+      <c r="O43" s="23"/>
+      <c r="P43" s="21" t="str">
+        <f aca="false">IF($A43="","",IF($K43&lt;=N($H43),MAX(0,2*N($H43)-$K43),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="23"/>
@@ -2458,6 +2731,12 @@
         <f aca="false">IF($A44="","",IF($K44&lt;=0,"Rupture",IF($K44&lt;=N($H44),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N44" s="23"/>
+      <c r="O44" s="23"/>
+      <c r="P44" s="21" t="str">
+        <f aca="false">IF($A44="","",IF($K44&lt;=N($H44),MAX(0,2*N($H44)-$K44),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="23"/>
@@ -2488,6 +2767,12 @@
         <f aca="false">IF($A45="","",IF($K45&lt;=0,"Rupture",IF($K45&lt;=N($H45),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N45" s="23"/>
+      <c r="O45" s="23"/>
+      <c r="P45" s="21" t="str">
+        <f aca="false">IF($A45="","",IF($K45&lt;=N($H45),MAX(0,2*N($H45)-$K45),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="23"/>
@@ -2518,6 +2803,12 @@
         <f aca="false">IF($A46="","",IF($K46&lt;=0,"Rupture",IF($K46&lt;=N($H46),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N46" s="23"/>
+      <c r="O46" s="23"/>
+      <c r="P46" s="21" t="str">
+        <f aca="false">IF($A46="","",IF($K46&lt;=N($H46),MAX(0,2*N($H46)-$K46),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="23"/>
@@ -2548,6 +2839,12 @@
         <f aca="false">IF($A47="","",IF($K47&lt;=0,"Rupture",IF($K47&lt;=N($H47),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N47" s="23"/>
+      <c r="O47" s="23"/>
+      <c r="P47" s="21" t="str">
+        <f aca="false">IF($A47="","",IF($K47&lt;=N($H47),MAX(0,2*N($H47)-$K47),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="23"/>
@@ -2578,6 +2875,12 @@
         <f aca="false">IF($A48="","",IF($K48&lt;=0,"Rupture",IF($K48&lt;=N($H48),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N48" s="23"/>
+      <c r="O48" s="23"/>
+      <c r="P48" s="21" t="str">
+        <f aca="false">IF($A48="","",IF($K48&lt;=N($H48),MAX(0,2*N($H48)-$K48),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="23"/>
@@ -2608,6 +2911,12 @@
         <f aca="false">IF($A49="","",IF($K49&lt;=0,"Rupture",IF($K49&lt;=N($H49),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N49" s="23"/>
+      <c r="O49" s="23"/>
+      <c r="P49" s="21" t="str">
+        <f aca="false">IF($A49="","",IF($K49&lt;=N($H49),MAX(0,2*N($H49)-$K49),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="23"/>
@@ -2638,6 +2947,12 @@
         <f aca="false">IF($A50="","",IF($K50&lt;=0,"Rupture",IF($K50&lt;=N($H50),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N50" s="23"/>
+      <c r="O50" s="23"/>
+      <c r="P50" s="21" t="str">
+        <f aca="false">IF($A50="","",IF($K50&lt;=N($H50),MAX(0,2*N($H50)-$K50),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="23"/>
@@ -2668,6 +2983,12 @@
         <f aca="false">IF($A51="","",IF($K51&lt;=0,"Rupture",IF($K51&lt;=N($H51),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N51" s="23"/>
+      <c r="O51" s="23"/>
+      <c r="P51" s="21" t="str">
+        <f aca="false">IF($A51="","",IF($K51&lt;=N($H51),MAX(0,2*N($H51)-$K51),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="23"/>
@@ -2698,6 +3019,12 @@
         <f aca="false">IF($A52="","",IF($K52&lt;=0,"Rupture",IF($K52&lt;=N($H52),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N52" s="23"/>
+      <c r="O52" s="23"/>
+      <c r="P52" s="21" t="str">
+        <f aca="false">IF($A52="","",IF($K52&lt;=N($H52),MAX(0,2*N($H52)-$K52),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="23"/>
@@ -2728,6 +3055,12 @@
         <f aca="false">IF($A53="","",IF($K53&lt;=0,"Rupture",IF($K53&lt;=N($H53),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N53" s="23"/>
+      <c r="O53" s="23"/>
+      <c r="P53" s="21" t="str">
+        <f aca="false">IF($A53="","",IF($K53&lt;=N($H53),MAX(0,2*N($H53)-$K53),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="23"/>
@@ -2758,6 +3091,12 @@
         <f aca="false">IF($A54="","",IF($K54&lt;=0,"Rupture",IF($K54&lt;=N($H54),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N54" s="23"/>
+      <c r="O54" s="23"/>
+      <c r="P54" s="21" t="str">
+        <f aca="false">IF($A54="","",IF($K54&lt;=N($H54),MAX(0,2*N($H54)-$K54),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="23"/>
@@ -2788,6 +3127,12 @@
         <f aca="false">IF($A55="","",IF($K55&lt;=0,"Rupture",IF($K55&lt;=N($H55),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N55" s="23"/>
+      <c r="O55" s="23"/>
+      <c r="P55" s="21" t="str">
+        <f aca="false">IF($A55="","",IF($K55&lt;=N($H55),MAX(0,2*N($H55)-$K55),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="23"/>
@@ -2818,6 +3163,12 @@
         <f aca="false">IF($A56="","",IF($K56&lt;=0,"Rupture",IF($K56&lt;=N($H56),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N56" s="23"/>
+      <c r="O56" s="23"/>
+      <c r="P56" s="21" t="str">
+        <f aca="false">IF($A56="","",IF($K56&lt;=N($H56),MAX(0,2*N($H56)-$K56),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="23"/>
@@ -2848,6 +3199,12 @@
         <f aca="false">IF($A57="","",IF($K57&lt;=0,"Rupture",IF($K57&lt;=N($H57),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N57" s="23"/>
+      <c r="O57" s="23"/>
+      <c r="P57" s="21" t="str">
+        <f aca="false">IF($A57="","",IF($K57&lt;=N($H57),MAX(0,2*N($H57)-$K57),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="23"/>
@@ -2878,6 +3235,12 @@
         <f aca="false">IF($A58="","",IF($K58&lt;=0,"Rupture",IF($K58&lt;=N($H58),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N58" s="23"/>
+      <c r="O58" s="23"/>
+      <c r="P58" s="21" t="str">
+        <f aca="false">IF($A58="","",IF($K58&lt;=N($H58),MAX(0,2*N($H58)-$K58),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="23"/>
@@ -2908,6 +3271,12 @@
         <f aca="false">IF($A59="","",IF($K59&lt;=0,"Rupture",IF($K59&lt;=N($H59),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N59" s="23"/>
+      <c r="O59" s="23"/>
+      <c r="P59" s="21" t="str">
+        <f aca="false">IF($A59="","",IF($K59&lt;=N($H59),MAX(0,2*N($H59)-$K59),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="23"/>
@@ -2938,6 +3307,12 @@
         <f aca="false">IF($A60="","",IF($K60&lt;=0,"Rupture",IF($K60&lt;=N($H60),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N60" s="23"/>
+      <c r="O60" s="23"/>
+      <c r="P60" s="21" t="str">
+        <f aca="false">IF($A60="","",IF($K60&lt;=N($H60),MAX(0,2*N($H60)-$K60),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="23"/>
@@ -2968,6 +3343,12 @@
         <f aca="false">IF($A61="","",IF($K61&lt;=0,"Rupture",IF($K61&lt;=N($H61),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N61" s="23"/>
+      <c r="O61" s="23"/>
+      <c r="P61" s="21" t="str">
+        <f aca="false">IF($A61="","",IF($K61&lt;=N($H61),MAX(0,2*N($H61)-$K61),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="23"/>
@@ -2998,6 +3379,12 @@
         <f aca="false">IF($A62="","",IF($K62&lt;=0,"Rupture",IF($K62&lt;=N($H62),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N62" s="23"/>
+      <c r="O62" s="23"/>
+      <c r="P62" s="21" t="str">
+        <f aca="false">IF($A62="","",IF($K62&lt;=N($H62),MAX(0,2*N($H62)-$K62),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="23"/>
@@ -3028,6 +3415,12 @@
         <f aca="false">IF($A63="","",IF($K63&lt;=0,"Rupture",IF($K63&lt;=N($H63),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N63" s="23"/>
+      <c r="O63" s="23"/>
+      <c r="P63" s="21" t="str">
+        <f aca="false">IF($A63="","",IF($K63&lt;=N($H63),MAX(0,2*N($H63)-$K63),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="23"/>
@@ -3058,6 +3451,12 @@
         <f aca="false">IF($A64="","",IF($K64&lt;=0,"Rupture",IF($K64&lt;=N($H64),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N64" s="23"/>
+      <c r="O64" s="23"/>
+      <c r="P64" s="21" t="str">
+        <f aca="false">IF($A64="","",IF($K64&lt;=N($H64),MAX(0,2*N($H64)-$K64),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="23"/>
@@ -3088,6 +3487,12 @@
         <f aca="false">IF($A65="","",IF($K65&lt;=0,"Rupture",IF($K65&lt;=N($H65),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N65" s="23"/>
+      <c r="O65" s="23"/>
+      <c r="P65" s="21" t="str">
+        <f aca="false">IF($A65="","",IF($K65&lt;=N($H65),MAX(0,2*N($H65)-$K65),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="23"/>
@@ -3118,6 +3523,12 @@
         <f aca="false">IF($A66="","",IF($K66&lt;=0,"Rupture",IF($K66&lt;=N($H66),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N66" s="23"/>
+      <c r="O66" s="23"/>
+      <c r="P66" s="21" t="str">
+        <f aca="false">IF($A66="","",IF($K66&lt;=N($H66),MAX(0,2*N($H66)-$K66),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="23"/>
@@ -3148,6 +3559,12 @@
         <f aca="false">IF($A67="","",IF($K67&lt;=0,"Rupture",IF($K67&lt;=N($H67),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N67" s="23"/>
+      <c r="O67" s="23"/>
+      <c r="P67" s="21" t="str">
+        <f aca="false">IF($A67="","",IF($K67&lt;=N($H67),MAX(0,2*N($H67)-$K67),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="23"/>
@@ -3178,6 +3595,12 @@
         <f aca="false">IF($A68="","",IF($K68&lt;=0,"Rupture",IF($K68&lt;=N($H68),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N68" s="23"/>
+      <c r="O68" s="23"/>
+      <c r="P68" s="21" t="str">
+        <f aca="false">IF($A68="","",IF($K68&lt;=N($H68),MAX(0,2*N($H68)-$K68),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="23"/>
@@ -3208,6 +3631,12 @@
         <f aca="false">IF($A69="","",IF($K69&lt;=0,"Rupture",IF($K69&lt;=N($H69),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N69" s="23"/>
+      <c r="O69" s="23"/>
+      <c r="P69" s="21" t="str">
+        <f aca="false">IF($A69="","",IF($K69&lt;=N($H69),MAX(0,2*N($H69)-$K69),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="23"/>
@@ -3238,6 +3667,12 @@
         <f aca="false">IF($A70="","",IF($K70&lt;=0,"Rupture",IF($K70&lt;=N($H70),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N70" s="23"/>
+      <c r="O70" s="23"/>
+      <c r="P70" s="21" t="str">
+        <f aca="false">IF($A70="","",IF($K70&lt;=N($H70),MAX(0,2*N($H70)-$K70),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="23"/>
@@ -3268,6 +3703,12 @@
         <f aca="false">IF($A71="","",IF($K71&lt;=0,"Rupture",IF($K71&lt;=N($H71),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N71" s="23"/>
+      <c r="O71" s="23"/>
+      <c r="P71" s="21" t="str">
+        <f aca="false">IF($A71="","",IF($K71&lt;=N($H71),MAX(0,2*N($H71)-$K71),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="23"/>
@@ -3298,6 +3739,12 @@
         <f aca="false">IF($A72="","",IF($K72&lt;=0,"Rupture",IF($K72&lt;=N($H72),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N72" s="23"/>
+      <c r="O72" s="23"/>
+      <c r="P72" s="21" t="str">
+        <f aca="false">IF($A72="","",IF($K72&lt;=N($H72),MAX(0,2*N($H72)-$K72),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="23"/>
@@ -3328,6 +3775,12 @@
         <f aca="false">IF($A73="","",IF($K73&lt;=0,"Rupture",IF($K73&lt;=N($H73),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N73" s="23"/>
+      <c r="O73" s="23"/>
+      <c r="P73" s="21" t="str">
+        <f aca="false">IF($A73="","",IF($K73&lt;=N($H73),MAX(0,2*N($H73)-$K73),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="23"/>
@@ -3358,6 +3811,12 @@
         <f aca="false">IF($A74="","",IF($K74&lt;=0,"Rupture",IF($K74&lt;=N($H74),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N74" s="23"/>
+      <c r="O74" s="23"/>
+      <c r="P74" s="21" t="str">
+        <f aca="false">IF($A74="","",IF($K74&lt;=N($H74),MAX(0,2*N($H74)-$K74),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="23"/>
@@ -3388,6 +3847,12 @@
         <f aca="false">IF($A75="","",IF($K75&lt;=0,"Rupture",IF($K75&lt;=N($H75),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N75" s="23"/>
+      <c r="O75" s="23"/>
+      <c r="P75" s="21" t="str">
+        <f aca="false">IF($A75="","",IF($K75&lt;=N($H75),MAX(0,2*N($H75)-$K75),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="23"/>
@@ -3418,6 +3883,12 @@
         <f aca="false">IF($A76="","",IF($K76&lt;=0,"Rupture",IF($K76&lt;=N($H76),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N76" s="23"/>
+      <c r="O76" s="23"/>
+      <c r="P76" s="21" t="str">
+        <f aca="false">IF($A76="","",IF($K76&lt;=N($H76),MAX(0,2*N($H76)-$K76),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="23"/>
@@ -3448,6 +3919,12 @@
         <f aca="false">IF($A77="","",IF($K77&lt;=0,"Rupture",IF($K77&lt;=N($H77),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N77" s="23"/>
+      <c r="O77" s="23"/>
+      <c r="P77" s="21" t="str">
+        <f aca="false">IF($A77="","",IF($K77&lt;=N($H77),MAX(0,2*N($H77)-$K77),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="23"/>
@@ -3478,6 +3955,12 @@
         <f aca="false">IF($A78="","",IF($K78&lt;=0,"Rupture",IF($K78&lt;=N($H78),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N78" s="23"/>
+      <c r="O78" s="23"/>
+      <c r="P78" s="21" t="str">
+        <f aca="false">IF($A78="","",IF($K78&lt;=N($H78),MAX(0,2*N($H78)-$K78),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="23"/>
@@ -3508,6 +3991,12 @@
         <f aca="false">IF($A79="","",IF($K79&lt;=0,"Rupture",IF($K79&lt;=N($H79),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N79" s="23"/>
+      <c r="O79" s="23"/>
+      <c r="P79" s="21" t="str">
+        <f aca="false">IF($A79="","",IF($K79&lt;=N($H79),MAX(0,2*N($H79)-$K79),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="23"/>
@@ -3538,6 +4027,12 @@
         <f aca="false">IF($A80="","",IF($K80&lt;=0,"Rupture",IF($K80&lt;=N($H80),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N80" s="23"/>
+      <c r="O80" s="23"/>
+      <c r="P80" s="21" t="str">
+        <f aca="false">IF($A80="","",IF($K80&lt;=N($H80),MAX(0,2*N($H80)-$K80),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="23"/>
@@ -3568,6 +4063,12 @@
         <f aca="false">IF($A81="","",IF($K81&lt;=0,"Rupture",IF($K81&lt;=N($H81),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N81" s="23"/>
+      <c r="O81" s="23"/>
+      <c r="P81" s="21" t="str">
+        <f aca="false">IF($A81="","",IF($K81&lt;=N($H81),MAX(0,2*N($H81)-$K81),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="23"/>
@@ -3598,6 +4099,12 @@
         <f aca="false">IF($A82="","",IF($K82&lt;=0,"Rupture",IF($K82&lt;=N($H82),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N82" s="23"/>
+      <c r="O82" s="23"/>
+      <c r="P82" s="21" t="str">
+        <f aca="false">IF($A82="","",IF($K82&lt;=N($H82),MAX(0,2*N($H82)-$K82),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="23"/>
@@ -3628,6 +4135,12 @@
         <f aca="false">IF($A83="","",IF($K83&lt;=0,"Rupture",IF($K83&lt;=N($H83),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N83" s="23"/>
+      <c r="O83" s="23"/>
+      <c r="P83" s="21" t="str">
+        <f aca="false">IF($A83="","",IF($K83&lt;=N($H83),MAX(0,2*N($H83)-$K83),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="23"/>
@@ -3658,6 +4171,12 @@
         <f aca="false">IF($A84="","",IF($K84&lt;=0,"Rupture",IF($K84&lt;=N($H84),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N84" s="23"/>
+      <c r="O84" s="23"/>
+      <c r="P84" s="21" t="str">
+        <f aca="false">IF($A84="","",IF($K84&lt;=N($H84),MAX(0,2*N($H84)-$K84),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="23"/>
@@ -3688,6 +4207,12 @@
         <f aca="false">IF($A85="","",IF($K85&lt;=0,"Rupture",IF($K85&lt;=N($H85),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N85" s="23"/>
+      <c r="O85" s="23"/>
+      <c r="P85" s="21" t="str">
+        <f aca="false">IF($A85="","",IF($K85&lt;=N($H85),MAX(0,2*N($H85)-$K85),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="23"/>
@@ -3718,6 +4243,12 @@
         <f aca="false">IF($A86="","",IF($K86&lt;=0,"Rupture",IF($K86&lt;=N($H86),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N86" s="23"/>
+      <c r="O86" s="23"/>
+      <c r="P86" s="21" t="str">
+        <f aca="false">IF($A86="","",IF($K86&lt;=N($H86),MAX(0,2*N($H86)-$K86),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="23"/>
@@ -3748,6 +4279,12 @@
         <f aca="false">IF($A87="","",IF($K87&lt;=0,"Rupture",IF($K87&lt;=N($H87),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N87" s="23"/>
+      <c r="O87" s="23"/>
+      <c r="P87" s="21" t="str">
+        <f aca="false">IF($A87="","",IF($K87&lt;=N($H87),MAX(0,2*N($H87)-$K87),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="23"/>
@@ -3778,6 +4315,12 @@
         <f aca="false">IF($A88="","",IF($K88&lt;=0,"Rupture",IF($K88&lt;=N($H88),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N88" s="23"/>
+      <c r="O88" s="23"/>
+      <c r="P88" s="21" t="str">
+        <f aca="false">IF($A88="","",IF($K88&lt;=N($H88),MAX(0,2*N($H88)-$K88),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="23"/>
@@ -3808,6 +4351,12 @@
         <f aca="false">IF($A89="","",IF($K89&lt;=0,"Rupture",IF($K89&lt;=N($H89),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N89" s="23"/>
+      <c r="O89" s="23"/>
+      <c r="P89" s="21" t="str">
+        <f aca="false">IF($A89="","",IF($K89&lt;=N($H89),MAX(0,2*N($H89)-$K89),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="23"/>
@@ -3838,6 +4387,12 @@
         <f aca="false">IF($A90="","",IF($K90&lt;=0,"Rupture",IF($K90&lt;=N($H90),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N90" s="23"/>
+      <c r="O90" s="23"/>
+      <c r="P90" s="21" t="str">
+        <f aca="false">IF($A90="","",IF($K90&lt;=N($H90),MAX(0,2*N($H90)-$K90),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="23"/>
@@ -3868,6 +4423,12 @@
         <f aca="false">IF($A91="","",IF($K91&lt;=0,"Rupture",IF($K91&lt;=N($H91),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N91" s="23"/>
+      <c r="O91" s="23"/>
+      <c r="P91" s="21" t="str">
+        <f aca="false">IF($A91="","",IF($K91&lt;=N($H91),MAX(0,2*N($H91)-$K91),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="23"/>
@@ -3898,6 +4459,12 @@
         <f aca="false">IF($A92="","",IF($K92&lt;=0,"Rupture",IF($K92&lt;=N($H92),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N92" s="23"/>
+      <c r="O92" s="23"/>
+      <c r="P92" s="21" t="str">
+        <f aca="false">IF($A92="","",IF($K92&lt;=N($H92),MAX(0,2*N($H92)-$K92),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="23"/>
@@ -3928,6 +4495,12 @@
         <f aca="false">IF($A93="","",IF($K93&lt;=0,"Rupture",IF($K93&lt;=N($H93),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N93" s="23"/>
+      <c r="O93" s="23"/>
+      <c r="P93" s="21" t="str">
+        <f aca="false">IF($A93="","",IF($K93&lt;=N($H93),MAX(0,2*N($H93)-$K93),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="23"/>
@@ -3958,6 +4531,12 @@
         <f aca="false">IF($A94="","",IF($K94&lt;=0,"Rupture",IF($K94&lt;=N($H94),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N94" s="23"/>
+      <c r="O94" s="23"/>
+      <c r="P94" s="21" t="str">
+        <f aca="false">IF($A94="","",IF($K94&lt;=N($H94),MAX(0,2*N($H94)-$K94),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="23"/>
@@ -3988,6 +4567,12 @@
         <f aca="false">IF($A95="","",IF($K95&lt;=0,"Rupture",IF($K95&lt;=N($H95),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N95" s="23"/>
+      <c r="O95" s="23"/>
+      <c r="P95" s="21" t="str">
+        <f aca="false">IF($A95="","",IF($K95&lt;=N($H95),MAX(0,2*N($H95)-$K95),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="23"/>
@@ -4018,6 +4603,12 @@
         <f aca="false">IF($A96="","",IF($K96&lt;=0,"Rupture",IF($K96&lt;=N($H96),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N96" s="23"/>
+      <c r="O96" s="23"/>
+      <c r="P96" s="21" t="str">
+        <f aca="false">IF($A96="","",IF($K96&lt;=N($H96),MAX(0,2*N($H96)-$K96),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="23"/>
@@ -4048,6 +4639,12 @@
         <f aca="false">IF($A97="","",IF($K97&lt;=0,"Rupture",IF($K97&lt;=N($H97),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N97" s="23"/>
+      <c r="O97" s="23"/>
+      <c r="P97" s="21" t="str">
+        <f aca="false">IF($A97="","",IF($K97&lt;=N($H97),MAX(0,2*N($H97)-$K97),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="23"/>
@@ -4078,6 +4675,12 @@
         <f aca="false">IF($A98="","",IF($K98&lt;=0,"Rupture",IF($K98&lt;=N($H98),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N98" s="23"/>
+      <c r="O98" s="23"/>
+      <c r="P98" s="21" t="str">
+        <f aca="false">IF($A98="","",IF($K98&lt;=N($H98),MAX(0,2*N($H98)-$K98),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="23"/>
@@ -4108,6 +4711,12 @@
         <f aca="false">IF($A99="","",IF($K99&lt;=0,"Rupture",IF($K99&lt;=N($H99),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N99" s="23"/>
+      <c r="O99" s="23"/>
+      <c r="P99" s="21" t="str">
+        <f aca="false">IF($A99="","",IF($K99&lt;=N($H99),MAX(0,2*N($H99)-$K99),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="23"/>
@@ -4138,6 +4747,12 @@
         <f aca="false">IF($A100="","",IF($K100&lt;=0,"Rupture",IF($K100&lt;=N($H100),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N100" s="23"/>
+      <c r="O100" s="23"/>
+      <c r="P100" s="21" t="str">
+        <f aca="false">IF($A100="","",IF($K100&lt;=N($H100),MAX(0,2*N($H100)-$K100),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="23"/>
@@ -4168,6 +4783,12 @@
         <f aca="false">IF($A101="","",IF($K101&lt;=0,"Rupture",IF($K101&lt;=N($H101),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N101" s="23"/>
+      <c r="O101" s="23"/>
+      <c r="P101" s="21" t="str">
+        <f aca="false">IF($A101="","",IF($K101&lt;=N($H101),MAX(0,2*N($H101)-$K101),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="23"/>
@@ -4198,6 +4819,12 @@
         <f aca="false">IF($A102="","",IF($K102&lt;=0,"Rupture",IF($K102&lt;=N($H102),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N102" s="23"/>
+      <c r="O102" s="23"/>
+      <c r="P102" s="21" t="str">
+        <f aca="false">IF($A102="","",IF($K102&lt;=N($H102),MAX(0,2*N($H102)-$K102),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="23"/>
@@ -4228,6 +4855,12 @@
         <f aca="false">IF($A103="","",IF($K103&lt;=0,"Rupture",IF($K103&lt;=N($H103),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N103" s="23"/>
+      <c r="O103" s="23"/>
+      <c r="P103" s="21" t="str">
+        <f aca="false">IF($A103="","",IF($K103&lt;=N($H103),MAX(0,2*N($H103)-$K103),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="23"/>
@@ -4258,6 +4891,12 @@
         <f aca="false">IF($A104="","",IF($K104&lt;=0,"Rupture",IF($K104&lt;=N($H104),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N104" s="23"/>
+      <c r="O104" s="23"/>
+      <c r="P104" s="21" t="str">
+        <f aca="false">IF($A104="","",IF($K104&lt;=N($H104),MAX(0,2*N($H104)-$K104),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="23"/>
@@ -4288,6 +4927,12 @@
         <f aca="false">IF($A105="","",IF($K105&lt;=0,"Rupture",IF($K105&lt;=N($H105),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N105" s="23"/>
+      <c r="O105" s="23"/>
+      <c r="P105" s="21" t="str">
+        <f aca="false">IF($A105="","",IF($K105&lt;=N($H105),MAX(0,2*N($H105)-$K105),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="23"/>
@@ -4318,6 +4963,12 @@
         <f aca="false">IF($A106="","",IF($K106&lt;=0,"Rupture",IF($K106&lt;=N($H106),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N106" s="23"/>
+      <c r="O106" s="23"/>
+      <c r="P106" s="21" t="str">
+        <f aca="false">IF($A106="","",IF($K106&lt;=N($H106),MAX(0,2*N($H106)-$K106),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="23"/>
@@ -4348,6 +4999,12 @@
         <f aca="false">IF($A107="","",IF($K107&lt;=0,"Rupture",IF($K107&lt;=N($H107),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N107" s="23"/>
+      <c r="O107" s="23"/>
+      <c r="P107" s="21" t="str">
+        <f aca="false">IF($A107="","",IF($K107&lt;=N($H107),MAX(0,2*N($H107)-$K107),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="23"/>
@@ -4378,6 +5035,12 @@
         <f aca="false">IF($A108="","",IF($K108&lt;=0,"Rupture",IF($K108&lt;=N($H108),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N108" s="23"/>
+      <c r="O108" s="23"/>
+      <c r="P108" s="21" t="str">
+        <f aca="false">IF($A108="","",IF($K108&lt;=N($H108),MAX(0,2*N($H108)-$K108),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="23"/>
@@ -4408,6 +5071,12 @@
         <f aca="false">IF($A109="","",IF($K109&lt;=0,"Rupture",IF($K109&lt;=N($H109),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N109" s="23"/>
+      <c r="O109" s="23"/>
+      <c r="P109" s="21" t="str">
+        <f aca="false">IF($A109="","",IF($K109&lt;=N($H109),MAX(0,2*N($H109)-$K109),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="23"/>
@@ -4438,6 +5107,12 @@
         <f aca="false">IF($A110="","",IF($K110&lt;=0,"Rupture",IF($K110&lt;=N($H110),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N110" s="23"/>
+      <c r="O110" s="23"/>
+      <c r="P110" s="21" t="str">
+        <f aca="false">IF($A110="","",IF($K110&lt;=N($H110),MAX(0,2*N($H110)-$K110),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="23"/>
@@ -4468,6 +5143,12 @@
         <f aca="false">IF($A111="","",IF($K111&lt;=0,"Rupture",IF($K111&lt;=N($H111),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N111" s="23"/>
+      <c r="O111" s="23"/>
+      <c r="P111" s="21" t="str">
+        <f aca="false">IF($A111="","",IF($K111&lt;=N($H111),MAX(0,2*N($H111)-$K111),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="23"/>
@@ -4498,6 +5179,12 @@
         <f aca="false">IF($A112="","",IF($K112&lt;=0,"Rupture",IF($K112&lt;=N($H112),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N112" s="23"/>
+      <c r="O112" s="23"/>
+      <c r="P112" s="21" t="str">
+        <f aca="false">IF($A112="","",IF($K112&lt;=N($H112),MAX(0,2*N($H112)-$K112),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="23"/>
@@ -4528,6 +5215,12 @@
         <f aca="false">IF($A113="","",IF($K113&lt;=0,"Rupture",IF($K113&lt;=N($H113),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N113" s="23"/>
+      <c r="O113" s="23"/>
+      <c r="P113" s="21" t="str">
+        <f aca="false">IF($A113="","",IF($K113&lt;=N($H113),MAX(0,2*N($H113)-$K113),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="23"/>
@@ -4558,6 +5251,12 @@
         <f aca="false">IF($A114="","",IF($K114&lt;=0,"Rupture",IF($K114&lt;=N($H114),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N114" s="23"/>
+      <c r="O114" s="23"/>
+      <c r="P114" s="21" t="str">
+        <f aca="false">IF($A114="","",IF($K114&lt;=N($H114),MAX(0,2*N($H114)-$K114),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="23"/>
@@ -4588,6 +5287,12 @@
         <f aca="false">IF($A115="","",IF($K115&lt;=0,"Rupture",IF($K115&lt;=N($H115),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N115" s="23"/>
+      <c r="O115" s="23"/>
+      <c r="P115" s="21" t="str">
+        <f aca="false">IF($A115="","",IF($K115&lt;=N($H115),MAX(0,2*N($H115)-$K115),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="23"/>
@@ -4618,6 +5323,12 @@
         <f aca="false">IF($A116="","",IF($K116&lt;=0,"Rupture",IF($K116&lt;=N($H116),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N116" s="23"/>
+      <c r="O116" s="23"/>
+      <c r="P116" s="21" t="str">
+        <f aca="false">IF($A116="","",IF($K116&lt;=N($H116),MAX(0,2*N($H116)-$K116),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="23"/>
@@ -4648,6 +5359,12 @@
         <f aca="false">IF($A117="","",IF($K117&lt;=0,"Rupture",IF($K117&lt;=N($H117),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N117" s="23"/>
+      <c r="O117" s="23"/>
+      <c r="P117" s="21" t="str">
+        <f aca="false">IF($A117="","",IF($K117&lt;=N($H117),MAX(0,2*N($H117)-$K117),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="23"/>
@@ -4678,6 +5395,12 @@
         <f aca="false">IF($A118="","",IF($K118&lt;=0,"Rupture",IF($K118&lt;=N($H118),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N118" s="23"/>
+      <c r="O118" s="23"/>
+      <c r="P118" s="21" t="str">
+        <f aca="false">IF($A118="","",IF($K118&lt;=N($H118),MAX(0,2*N($H118)-$K118),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="23"/>
@@ -4708,6 +5431,12 @@
         <f aca="false">IF($A119="","",IF($K119&lt;=0,"Rupture",IF($K119&lt;=N($H119),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N119" s="23"/>
+      <c r="O119" s="23"/>
+      <c r="P119" s="21" t="str">
+        <f aca="false">IF($A119="","",IF($K119&lt;=N($H119),MAX(0,2*N($H119)-$K119),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="23"/>
@@ -4738,6 +5467,12 @@
         <f aca="false">IF($A120="","",IF($K120&lt;=0,"Rupture",IF($K120&lt;=N($H120),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N120" s="23"/>
+      <c r="O120" s="23"/>
+      <c r="P120" s="21" t="str">
+        <f aca="false">IF($A120="","",IF($K120&lt;=N($H120),MAX(0,2*N($H120)-$K120),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="23"/>
@@ -4768,6 +5503,12 @@
         <f aca="false">IF($A121="","",IF($K121&lt;=0,"Rupture",IF($K121&lt;=N($H121),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N121" s="23"/>
+      <c r="O121" s="23"/>
+      <c r="P121" s="21" t="str">
+        <f aca="false">IF($A121="","",IF($K121&lt;=N($H121),MAX(0,2*N($H121)-$K121),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="23"/>
@@ -4798,6 +5539,12 @@
         <f aca="false">IF($A122="","",IF($K122&lt;=0,"Rupture",IF($K122&lt;=N($H122),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N122" s="23"/>
+      <c r="O122" s="23"/>
+      <c r="P122" s="21" t="str">
+        <f aca="false">IF($A122="","",IF($K122&lt;=N($H122),MAX(0,2*N($H122)-$K122),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="23"/>
@@ -4828,6 +5575,12 @@
         <f aca="false">IF($A123="","",IF($K123&lt;=0,"Rupture",IF($K123&lt;=N($H123),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N123" s="23"/>
+      <c r="O123" s="23"/>
+      <c r="P123" s="21" t="str">
+        <f aca="false">IF($A123="","",IF($K123&lt;=N($H123),MAX(0,2*N($H123)-$K123),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="23"/>
@@ -4858,6 +5611,12 @@
         <f aca="false">IF($A124="","",IF($K124&lt;=0,"Rupture",IF($K124&lt;=N($H124),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N124" s="23"/>
+      <c r="O124" s="23"/>
+      <c r="P124" s="21" t="str">
+        <f aca="false">IF($A124="","",IF($K124&lt;=N($H124),MAX(0,2*N($H124)-$K124),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="23"/>
@@ -4888,6 +5647,12 @@
         <f aca="false">IF($A125="","",IF($K125&lt;=0,"Rupture",IF($K125&lt;=N($H125),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N125" s="23"/>
+      <c r="O125" s="23"/>
+      <c r="P125" s="21" t="str">
+        <f aca="false">IF($A125="","",IF($K125&lt;=N($H125),MAX(0,2*N($H125)-$K125),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="23"/>
@@ -4918,6 +5683,12 @@
         <f aca="false">IF($A126="","",IF($K126&lt;=0,"Rupture",IF($K126&lt;=N($H126),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N126" s="23"/>
+      <c r="O126" s="23"/>
+      <c r="P126" s="21" t="str">
+        <f aca="false">IF($A126="","",IF($K126&lt;=N($H126),MAX(0,2*N($H126)-$K126),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="23"/>
@@ -4948,6 +5719,12 @@
         <f aca="false">IF($A127="","",IF($K127&lt;=0,"Rupture",IF($K127&lt;=N($H127),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N127" s="23"/>
+      <c r="O127" s="23"/>
+      <c r="P127" s="21" t="str">
+        <f aca="false">IF($A127="","",IF($K127&lt;=N($H127),MAX(0,2*N($H127)-$K127),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="23"/>
@@ -4978,6 +5755,12 @@
         <f aca="false">IF($A128="","",IF($K128&lt;=0,"Rupture",IF($K128&lt;=N($H128),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N128" s="23"/>
+      <c r="O128" s="23"/>
+      <c r="P128" s="21" t="str">
+        <f aca="false">IF($A128="","",IF($K128&lt;=N($H128),MAX(0,2*N($H128)-$K128),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="23"/>
@@ -5008,6 +5791,12 @@
         <f aca="false">IF($A129="","",IF($K129&lt;=0,"Rupture",IF($K129&lt;=N($H129),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N129" s="23"/>
+      <c r="O129" s="23"/>
+      <c r="P129" s="21" t="str">
+        <f aca="false">IF($A129="","",IF($K129&lt;=N($H129),MAX(0,2*N($H129)-$K129),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="23"/>
@@ -5038,6 +5827,12 @@
         <f aca="false">IF($A130="","",IF($K130&lt;=0,"Rupture",IF($K130&lt;=N($H130),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N130" s="23"/>
+      <c r="O130" s="23"/>
+      <c r="P130" s="21" t="str">
+        <f aca="false">IF($A130="","",IF($K130&lt;=N($H130),MAX(0,2*N($H130)-$K130),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="23"/>
@@ -5068,6 +5863,12 @@
         <f aca="false">IF($A131="","",IF($K131&lt;=0,"Rupture",IF($K131&lt;=N($H131),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N131" s="23"/>
+      <c r="O131" s="23"/>
+      <c r="P131" s="21" t="str">
+        <f aca="false">IF($A131="","",IF($K131&lt;=N($H131),MAX(0,2*N($H131)-$K131),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="23"/>
@@ -5098,6 +5899,12 @@
         <f aca="false">IF($A132="","",IF($K132&lt;=0,"Rupture",IF($K132&lt;=N($H132),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N132" s="23"/>
+      <c r="O132" s="23"/>
+      <c r="P132" s="21" t="str">
+        <f aca="false">IF($A132="","",IF($K132&lt;=N($H132),MAX(0,2*N($H132)-$K132),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="23"/>
@@ -5128,6 +5935,12 @@
         <f aca="false">IF($A133="","",IF($K133&lt;=0,"Rupture",IF($K133&lt;=N($H133),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N133" s="23"/>
+      <c r="O133" s="23"/>
+      <c r="P133" s="21" t="str">
+        <f aca="false">IF($A133="","",IF($K133&lt;=N($H133),MAX(0,2*N($H133)-$K133),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="23"/>
@@ -5158,6 +5971,12 @@
         <f aca="false">IF($A134="","",IF($K134&lt;=0,"Rupture",IF($K134&lt;=N($H134),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N134" s="23"/>
+      <c r="O134" s="23"/>
+      <c r="P134" s="21" t="str">
+        <f aca="false">IF($A134="","",IF($K134&lt;=N($H134),MAX(0,2*N($H134)-$K134),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="23"/>
@@ -5188,6 +6007,12 @@
         <f aca="false">IF($A135="","",IF($K135&lt;=0,"Rupture",IF($K135&lt;=N($H135),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N135" s="23"/>
+      <c r="O135" s="23"/>
+      <c r="P135" s="21" t="str">
+        <f aca="false">IF($A135="","",IF($K135&lt;=N($H135),MAX(0,2*N($H135)-$K135),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="23"/>
@@ -5218,6 +6043,12 @@
         <f aca="false">IF($A136="","",IF($K136&lt;=0,"Rupture",IF($K136&lt;=N($H136),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N136" s="23"/>
+      <c r="O136" s="23"/>
+      <c r="P136" s="21" t="str">
+        <f aca="false">IF($A136="","",IF($K136&lt;=N($H136),MAX(0,2*N($H136)-$K136),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="23"/>
@@ -5248,6 +6079,12 @@
         <f aca="false">IF($A137="","",IF($K137&lt;=0,"Rupture",IF($K137&lt;=N($H137),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N137" s="23"/>
+      <c r="O137" s="23"/>
+      <c r="P137" s="21" t="str">
+        <f aca="false">IF($A137="","",IF($K137&lt;=N($H137),MAX(0,2*N($H137)-$K137),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="23"/>
@@ -5278,6 +6115,12 @@
         <f aca="false">IF($A138="","",IF($K138&lt;=0,"Rupture",IF($K138&lt;=N($H138),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N138" s="23"/>
+      <c r="O138" s="23"/>
+      <c r="P138" s="21" t="str">
+        <f aca="false">IF($A138="","",IF($K138&lt;=N($H138),MAX(0,2*N($H138)-$K138),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="23"/>
@@ -5308,6 +6151,12 @@
         <f aca="false">IF($A139="","",IF($K139&lt;=0,"Rupture",IF($K139&lt;=N($H139),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N139" s="23"/>
+      <c r="O139" s="23"/>
+      <c r="P139" s="21" t="str">
+        <f aca="false">IF($A139="","",IF($K139&lt;=N($H139),MAX(0,2*N($H139)-$K139),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="23"/>
@@ -5338,6 +6187,12 @@
         <f aca="false">IF($A140="","",IF($K140&lt;=0,"Rupture",IF($K140&lt;=N($H140),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N140" s="23"/>
+      <c r="O140" s="23"/>
+      <c r="P140" s="21" t="str">
+        <f aca="false">IF($A140="","",IF($K140&lt;=N($H140),MAX(0,2*N($H140)-$K140),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="23"/>
@@ -5368,6 +6223,12 @@
         <f aca="false">IF($A141="","",IF($K141&lt;=0,"Rupture",IF($K141&lt;=N($H141),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N141" s="23"/>
+      <c r="O141" s="23"/>
+      <c r="P141" s="21" t="str">
+        <f aca="false">IF($A141="","",IF($K141&lt;=N($H141),MAX(0,2*N($H141)-$K141),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="23"/>
@@ -5398,6 +6259,12 @@
         <f aca="false">IF($A142="","",IF($K142&lt;=0,"Rupture",IF($K142&lt;=N($H142),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N142" s="23"/>
+      <c r="O142" s="23"/>
+      <c r="P142" s="21" t="str">
+        <f aca="false">IF($A142="","",IF($K142&lt;=N($H142),MAX(0,2*N($H142)-$K142),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="23"/>
@@ -5428,6 +6295,12 @@
         <f aca="false">IF($A143="","",IF($K143&lt;=0,"Rupture",IF($K143&lt;=N($H143),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N143" s="23"/>
+      <c r="O143" s="23"/>
+      <c r="P143" s="21" t="str">
+        <f aca="false">IF($A143="","",IF($K143&lt;=N($H143),MAX(0,2*N($H143)-$K143),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="23"/>
@@ -5458,6 +6331,12 @@
         <f aca="false">IF($A144="","",IF($K144&lt;=0,"Rupture",IF($K144&lt;=N($H144),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N144" s="23"/>
+      <c r="O144" s="23"/>
+      <c r="P144" s="21" t="str">
+        <f aca="false">IF($A144="","",IF($K144&lt;=N($H144),MAX(0,2*N($H144)-$K144),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="23"/>
@@ -5488,6 +6367,12 @@
         <f aca="false">IF($A145="","",IF($K145&lt;=0,"Rupture",IF($K145&lt;=N($H145),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N145" s="23"/>
+      <c r="O145" s="23"/>
+      <c r="P145" s="21" t="str">
+        <f aca="false">IF($A145="","",IF($K145&lt;=N($H145),MAX(0,2*N($H145)-$K145),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="23"/>
@@ -5518,6 +6403,12 @@
         <f aca="false">IF($A146="","",IF($K146&lt;=0,"Rupture",IF($K146&lt;=N($H146),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N146" s="23"/>
+      <c r="O146" s="23"/>
+      <c r="P146" s="21" t="str">
+        <f aca="false">IF($A146="","",IF($K146&lt;=N($H146),MAX(0,2*N($H146)-$K146),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="23"/>
@@ -5548,6 +6439,12 @@
         <f aca="false">IF($A147="","",IF($K147&lt;=0,"Rupture",IF($K147&lt;=N($H147),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N147" s="23"/>
+      <c r="O147" s="23"/>
+      <c r="P147" s="21" t="str">
+        <f aca="false">IF($A147="","",IF($K147&lt;=N($H147),MAX(0,2*N($H147)-$K147),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="23"/>
@@ -5578,6 +6475,12 @@
         <f aca="false">IF($A148="","",IF($K148&lt;=0,"Rupture",IF($K148&lt;=N($H148),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N148" s="23"/>
+      <c r="O148" s="23"/>
+      <c r="P148" s="21" t="str">
+        <f aca="false">IF($A148="","",IF($K148&lt;=N($H148),MAX(0,2*N($H148)-$K148),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="23"/>
@@ -5608,6 +6511,12 @@
         <f aca="false">IF($A149="","",IF($K149&lt;=0,"Rupture",IF($K149&lt;=N($H149),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N149" s="23"/>
+      <c r="O149" s="23"/>
+      <c r="P149" s="21" t="str">
+        <f aca="false">IF($A149="","",IF($K149&lt;=N($H149),MAX(0,2*N($H149)-$K149),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="23"/>
@@ -5638,6 +6547,12 @@
         <f aca="false">IF($A150="","",IF($K150&lt;=0,"Rupture",IF($K150&lt;=N($H150),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N150" s="23"/>
+      <c r="O150" s="23"/>
+      <c r="P150" s="21" t="str">
+        <f aca="false">IF($A150="","",IF($K150&lt;=N($H150),MAX(0,2*N($H150)-$K150),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="23"/>
@@ -5668,6 +6583,12 @@
         <f aca="false">IF($A151="","",IF($K151&lt;=0,"Rupture",IF($K151&lt;=N($H151),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N151" s="23"/>
+      <c r="O151" s="23"/>
+      <c r="P151" s="21" t="str">
+        <f aca="false">IF($A151="","",IF($K151&lt;=N($H151),MAX(0,2*N($H151)-$K151),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="23"/>
@@ -5698,6 +6619,12 @@
         <f aca="false">IF($A152="","",IF($K152&lt;=0,"Rupture",IF($K152&lt;=N($H152),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N152" s="23"/>
+      <c r="O152" s="23"/>
+      <c r="P152" s="21" t="str">
+        <f aca="false">IF($A152="","",IF($K152&lt;=N($H152),MAX(0,2*N($H152)-$K152),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="23"/>
@@ -5728,6 +6655,12 @@
         <f aca="false">IF($A153="","",IF($K153&lt;=0,"Rupture",IF($K153&lt;=N($H153),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N153" s="23"/>
+      <c r="O153" s="23"/>
+      <c r="P153" s="21" t="str">
+        <f aca="false">IF($A153="","",IF($K153&lt;=N($H153),MAX(0,2*N($H153)-$K153),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="23"/>
@@ -5758,6 +6691,12 @@
         <f aca="false">IF($A154="","",IF($K154&lt;=0,"Rupture",IF($K154&lt;=N($H154),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N154" s="23"/>
+      <c r="O154" s="23"/>
+      <c r="P154" s="21" t="str">
+        <f aca="false">IF($A154="","",IF($K154&lt;=N($H154),MAX(0,2*N($H154)-$K154),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="23"/>
@@ -5788,6 +6727,12 @@
         <f aca="false">IF($A155="","",IF($K155&lt;=0,"Rupture",IF($K155&lt;=N($H155),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N155" s="23"/>
+      <c r="O155" s="23"/>
+      <c r="P155" s="21" t="str">
+        <f aca="false">IF($A155="","",IF($K155&lt;=N($H155),MAX(0,2*N($H155)-$K155),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="23"/>
@@ -5818,6 +6763,12 @@
         <f aca="false">IF($A156="","",IF($K156&lt;=0,"Rupture",IF($K156&lt;=N($H156),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N156" s="23"/>
+      <c r="O156" s="23"/>
+      <c r="P156" s="21" t="str">
+        <f aca="false">IF($A156="","",IF($K156&lt;=N($H156),MAX(0,2*N($H156)-$K156),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="23"/>
@@ -5848,6 +6799,12 @@
         <f aca="false">IF($A157="","",IF($K157&lt;=0,"Rupture",IF($K157&lt;=N($H157),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N157" s="23"/>
+      <c r="O157" s="23"/>
+      <c r="P157" s="21" t="str">
+        <f aca="false">IF($A157="","",IF($K157&lt;=N($H157),MAX(0,2*N($H157)-$K157),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="23"/>
@@ -5878,6 +6835,12 @@
         <f aca="false">IF($A158="","",IF($K158&lt;=0,"Rupture",IF($K158&lt;=N($H158),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N158" s="23"/>
+      <c r="O158" s="23"/>
+      <c r="P158" s="21" t="str">
+        <f aca="false">IF($A158="","",IF($K158&lt;=N($H158),MAX(0,2*N($H158)-$K158),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="23"/>
@@ -5908,6 +6871,12 @@
         <f aca="false">IF($A159="","",IF($K159&lt;=0,"Rupture",IF($K159&lt;=N($H159),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N159" s="23"/>
+      <c r="O159" s="23"/>
+      <c r="P159" s="21" t="str">
+        <f aca="false">IF($A159="","",IF($K159&lt;=N($H159),MAX(0,2*N($H159)-$K159),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="23"/>
@@ -5938,6 +6907,12 @@
         <f aca="false">IF($A160="","",IF($K160&lt;=0,"Rupture",IF($K160&lt;=N($H160),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N160" s="23"/>
+      <c r="O160" s="23"/>
+      <c r="P160" s="21" t="str">
+        <f aca="false">IF($A160="","",IF($K160&lt;=N($H160),MAX(0,2*N($H160)-$K160),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="23"/>
@@ -5968,6 +6943,12 @@
         <f aca="false">IF($A161="","",IF($K161&lt;=0,"Rupture",IF($K161&lt;=N($H161),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N161" s="23"/>
+      <c r="O161" s="23"/>
+      <c r="P161" s="21" t="str">
+        <f aca="false">IF($A161="","",IF($K161&lt;=N($H161),MAX(0,2*N($H161)-$K161),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="23"/>
@@ -5998,6 +6979,12 @@
         <f aca="false">IF($A162="","",IF($K162&lt;=0,"Rupture",IF($K162&lt;=N($H162),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N162" s="23"/>
+      <c r="O162" s="23"/>
+      <c r="P162" s="21" t="str">
+        <f aca="false">IF($A162="","",IF($K162&lt;=N($H162),MAX(0,2*N($H162)-$K162),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="23"/>
@@ -6028,6 +7015,12 @@
         <f aca="false">IF($A163="","",IF($K163&lt;=0,"Rupture",IF($K163&lt;=N($H163),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N163" s="23"/>
+      <c r="O163" s="23"/>
+      <c r="P163" s="21" t="str">
+        <f aca="false">IF($A163="","",IF($K163&lt;=N($H163),MAX(0,2*N($H163)-$K163),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="23"/>
@@ -6058,6 +7051,12 @@
         <f aca="false">IF($A164="","",IF($K164&lt;=0,"Rupture",IF($K164&lt;=N($H164),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N164" s="23"/>
+      <c r="O164" s="23"/>
+      <c r="P164" s="21" t="str">
+        <f aca="false">IF($A164="","",IF($K164&lt;=N($H164),MAX(0,2*N($H164)-$K164),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="23"/>
@@ -6088,6 +7087,12 @@
         <f aca="false">IF($A165="","",IF($K165&lt;=0,"Rupture",IF($K165&lt;=N($H165),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N165" s="23"/>
+      <c r="O165" s="23"/>
+      <c r="P165" s="21" t="str">
+        <f aca="false">IF($A165="","",IF($K165&lt;=N($H165),MAX(0,2*N($H165)-$K165),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="23"/>
@@ -6118,6 +7123,12 @@
         <f aca="false">IF($A166="","",IF($K166&lt;=0,"Rupture",IF($K166&lt;=N($H166),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N166" s="23"/>
+      <c r="O166" s="23"/>
+      <c r="P166" s="21" t="str">
+        <f aca="false">IF($A166="","",IF($K166&lt;=N($H166),MAX(0,2*N($H166)-$K166),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="23"/>
@@ -6148,6 +7159,12 @@
         <f aca="false">IF($A167="","",IF($K167&lt;=0,"Rupture",IF($K167&lt;=N($H167),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N167" s="23"/>
+      <c r="O167" s="23"/>
+      <c r="P167" s="21" t="str">
+        <f aca="false">IF($A167="","",IF($K167&lt;=N($H167),MAX(0,2*N($H167)-$K167),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="23"/>
@@ -6178,6 +7195,12 @@
         <f aca="false">IF($A168="","",IF($K168&lt;=0,"Rupture",IF($K168&lt;=N($H168),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N168" s="23"/>
+      <c r="O168" s="23"/>
+      <c r="P168" s="21" t="str">
+        <f aca="false">IF($A168="","",IF($K168&lt;=N($H168),MAX(0,2*N($H168)-$K168),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="23"/>
@@ -6208,6 +7231,12 @@
         <f aca="false">IF($A169="","",IF($K169&lt;=0,"Rupture",IF($K169&lt;=N($H169),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N169" s="23"/>
+      <c r="O169" s="23"/>
+      <c r="P169" s="21" t="str">
+        <f aca="false">IF($A169="","",IF($K169&lt;=N($H169),MAX(0,2*N($H169)-$K169),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="23"/>
@@ -6238,6 +7267,12 @@
         <f aca="false">IF($A170="","",IF($K170&lt;=0,"Rupture",IF($K170&lt;=N($H170),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N170" s="23"/>
+      <c r="O170" s="23"/>
+      <c r="P170" s="21" t="str">
+        <f aca="false">IF($A170="","",IF($K170&lt;=N($H170),MAX(0,2*N($H170)-$K170),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="23"/>
@@ -6268,6 +7303,12 @@
         <f aca="false">IF($A171="","",IF($K171&lt;=0,"Rupture",IF($K171&lt;=N($H171),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N171" s="23"/>
+      <c r="O171" s="23"/>
+      <c r="P171" s="21" t="str">
+        <f aca="false">IF($A171="","",IF($K171&lt;=N($H171),MAX(0,2*N($H171)-$K171),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="23"/>
@@ -6298,6 +7339,12 @@
         <f aca="false">IF($A172="","",IF($K172&lt;=0,"Rupture",IF($K172&lt;=N($H172),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N172" s="23"/>
+      <c r="O172" s="23"/>
+      <c r="P172" s="21" t="str">
+        <f aca="false">IF($A172="","",IF($K172&lt;=N($H172),MAX(0,2*N($H172)-$K172),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="23"/>
@@ -6328,6 +7375,12 @@
         <f aca="false">IF($A173="","",IF($K173&lt;=0,"Rupture",IF($K173&lt;=N($H173),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N173" s="23"/>
+      <c r="O173" s="23"/>
+      <c r="P173" s="21" t="str">
+        <f aca="false">IF($A173="","",IF($K173&lt;=N($H173),MAX(0,2*N($H173)-$K173),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="23"/>
@@ -6358,6 +7411,12 @@
         <f aca="false">IF($A174="","",IF($K174&lt;=0,"Rupture",IF($K174&lt;=N($H174),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N174" s="23"/>
+      <c r="O174" s="23"/>
+      <c r="P174" s="21" t="str">
+        <f aca="false">IF($A174="","",IF($K174&lt;=N($H174),MAX(0,2*N($H174)-$K174),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="23"/>
@@ -6388,6 +7447,12 @@
         <f aca="false">IF($A175="","",IF($K175&lt;=0,"Rupture",IF($K175&lt;=N($H175),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N175" s="23"/>
+      <c r="O175" s="23"/>
+      <c r="P175" s="21" t="str">
+        <f aca="false">IF($A175="","",IF($K175&lt;=N($H175),MAX(0,2*N($H175)-$K175),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="23"/>
@@ -6418,6 +7483,12 @@
         <f aca="false">IF($A176="","",IF($K176&lt;=0,"Rupture",IF($K176&lt;=N($H176),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N176" s="23"/>
+      <c r="O176" s="23"/>
+      <c r="P176" s="21" t="str">
+        <f aca="false">IF($A176="","",IF($K176&lt;=N($H176),MAX(0,2*N($H176)-$K176),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="23"/>
@@ -6448,6 +7519,12 @@
         <f aca="false">IF($A177="","",IF($K177&lt;=0,"Rupture",IF($K177&lt;=N($H177),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N177" s="23"/>
+      <c r="O177" s="23"/>
+      <c r="P177" s="21" t="str">
+        <f aca="false">IF($A177="","",IF($K177&lt;=N($H177),MAX(0,2*N($H177)-$K177),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="23"/>
@@ -6478,6 +7555,12 @@
         <f aca="false">IF($A178="","",IF($K178&lt;=0,"Rupture",IF($K178&lt;=N($H178),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N178" s="23"/>
+      <c r="O178" s="23"/>
+      <c r="P178" s="21" t="str">
+        <f aca="false">IF($A178="","",IF($K178&lt;=N($H178),MAX(0,2*N($H178)-$K178),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="23"/>
@@ -6508,6 +7591,12 @@
         <f aca="false">IF($A179="","",IF($K179&lt;=0,"Rupture",IF($K179&lt;=N($H179),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N179" s="23"/>
+      <c r="O179" s="23"/>
+      <c r="P179" s="21" t="str">
+        <f aca="false">IF($A179="","",IF($K179&lt;=N($H179),MAX(0,2*N($H179)-$K179),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="23"/>
@@ -6538,6 +7627,12 @@
         <f aca="false">IF($A180="","",IF($K180&lt;=0,"Rupture",IF($K180&lt;=N($H180),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N180" s="23"/>
+      <c r="O180" s="23"/>
+      <c r="P180" s="21" t="str">
+        <f aca="false">IF($A180="","",IF($K180&lt;=N($H180),MAX(0,2*N($H180)-$K180),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="23"/>
@@ -6568,6 +7663,12 @@
         <f aca="false">IF($A181="","",IF($K181&lt;=0,"Rupture",IF($K181&lt;=N($H181),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N181" s="23"/>
+      <c r="O181" s="23"/>
+      <c r="P181" s="21" t="str">
+        <f aca="false">IF($A181="","",IF($K181&lt;=N($H181),MAX(0,2*N($H181)-$K181),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="23"/>
@@ -6598,6 +7699,12 @@
         <f aca="false">IF($A182="","",IF($K182&lt;=0,"Rupture",IF($K182&lt;=N($H182),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N182" s="23"/>
+      <c r="O182" s="23"/>
+      <c r="P182" s="21" t="str">
+        <f aca="false">IF($A182="","",IF($K182&lt;=N($H182),MAX(0,2*N($H182)-$K182),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="23"/>
@@ -6628,6 +7735,12 @@
         <f aca="false">IF($A183="","",IF($K183&lt;=0,"Rupture",IF($K183&lt;=N($H183),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N183" s="23"/>
+      <c r="O183" s="23"/>
+      <c r="P183" s="21" t="str">
+        <f aca="false">IF($A183="","",IF($K183&lt;=N($H183),MAX(0,2*N($H183)-$K183),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="23"/>
@@ -6658,6 +7771,12 @@
         <f aca="false">IF($A184="","",IF($K184&lt;=0,"Rupture",IF($K184&lt;=N($H184),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N184" s="23"/>
+      <c r="O184" s="23"/>
+      <c r="P184" s="21" t="str">
+        <f aca="false">IF($A184="","",IF($K184&lt;=N($H184),MAX(0,2*N($H184)-$K184),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="23"/>
@@ -6688,6 +7807,12 @@
         <f aca="false">IF($A185="","",IF($K185&lt;=0,"Rupture",IF($K185&lt;=N($H185),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N185" s="23"/>
+      <c r="O185" s="23"/>
+      <c r="P185" s="21" t="str">
+        <f aca="false">IF($A185="","",IF($K185&lt;=N($H185),MAX(0,2*N($H185)-$K185),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="23"/>
@@ -6718,6 +7843,12 @@
         <f aca="false">IF($A186="","",IF($K186&lt;=0,"Rupture",IF($K186&lt;=N($H186),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N186" s="23"/>
+      <c r="O186" s="23"/>
+      <c r="P186" s="21" t="str">
+        <f aca="false">IF($A186="","",IF($K186&lt;=N($H186),MAX(0,2*N($H186)-$K186),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="23"/>
@@ -6748,6 +7879,12 @@
         <f aca="false">IF($A187="","",IF($K187&lt;=0,"Rupture",IF($K187&lt;=N($H187),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N187" s="23"/>
+      <c r="O187" s="23"/>
+      <c r="P187" s="21" t="str">
+        <f aca="false">IF($A187="","",IF($K187&lt;=N($H187),MAX(0,2*N($H187)-$K187),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="23"/>
@@ -6778,6 +7915,12 @@
         <f aca="false">IF($A188="","",IF($K188&lt;=0,"Rupture",IF($K188&lt;=N($H188),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N188" s="23"/>
+      <c r="O188" s="23"/>
+      <c r="P188" s="21" t="str">
+        <f aca="false">IF($A188="","",IF($K188&lt;=N($H188),MAX(0,2*N($H188)-$K188),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="23"/>
@@ -6808,6 +7951,12 @@
         <f aca="false">IF($A189="","",IF($K189&lt;=0,"Rupture",IF($K189&lt;=N($H189),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N189" s="23"/>
+      <c r="O189" s="23"/>
+      <c r="P189" s="21" t="str">
+        <f aca="false">IF($A189="","",IF($K189&lt;=N($H189),MAX(0,2*N($H189)-$K189),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="23"/>
@@ -6838,6 +7987,12 @@
         <f aca="false">IF($A190="","",IF($K190&lt;=0,"Rupture",IF($K190&lt;=N($H190),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N190" s="23"/>
+      <c r="O190" s="23"/>
+      <c r="P190" s="21" t="str">
+        <f aca="false">IF($A190="","",IF($K190&lt;=N($H190),MAX(0,2*N($H190)-$K190),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="23"/>
@@ -6868,6 +8023,12 @@
         <f aca="false">IF($A191="","",IF($K191&lt;=0,"Rupture",IF($K191&lt;=N($H191),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N191" s="23"/>
+      <c r="O191" s="23"/>
+      <c r="P191" s="21" t="str">
+        <f aca="false">IF($A191="","",IF($K191&lt;=N($H191),MAX(0,2*N($H191)-$K191),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="23"/>
@@ -6898,6 +8059,12 @@
         <f aca="false">IF($A192="","",IF($K192&lt;=0,"Rupture",IF($K192&lt;=N($H192),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N192" s="23"/>
+      <c r="O192" s="23"/>
+      <c r="P192" s="21" t="str">
+        <f aca="false">IF($A192="","",IF($K192&lt;=N($H192),MAX(0,2*N($H192)-$K192),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="23"/>
@@ -6928,6 +8095,12 @@
         <f aca="false">IF($A193="","",IF($K193&lt;=0,"Rupture",IF($K193&lt;=N($H193),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N193" s="23"/>
+      <c r="O193" s="23"/>
+      <c r="P193" s="21" t="str">
+        <f aca="false">IF($A193="","",IF($K193&lt;=N($H193),MAX(0,2*N($H193)-$K193),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="23"/>
@@ -6958,6 +8131,12 @@
         <f aca="false">IF($A194="","",IF($K194&lt;=0,"Rupture",IF($K194&lt;=N($H194),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N194" s="23"/>
+      <c r="O194" s="23"/>
+      <c r="P194" s="21" t="str">
+        <f aca="false">IF($A194="","",IF($K194&lt;=N($H194),MAX(0,2*N($H194)-$K194),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="23"/>
@@ -6988,6 +8167,12 @@
         <f aca="false">IF($A195="","",IF($K195&lt;=0,"Rupture",IF($K195&lt;=N($H195),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N195" s="23"/>
+      <c r="O195" s="23"/>
+      <c r="P195" s="21" t="str">
+        <f aca="false">IF($A195="","",IF($K195&lt;=N($H195),MAX(0,2*N($H195)-$K195),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="23"/>
@@ -7018,6 +8203,12 @@
         <f aca="false">IF($A196="","",IF($K196&lt;=0,"Rupture",IF($K196&lt;=N($H196),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N196" s="23"/>
+      <c r="O196" s="23"/>
+      <c r="P196" s="21" t="str">
+        <f aca="false">IF($A196="","",IF($K196&lt;=N($H196),MAX(0,2*N($H196)-$K196),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="23"/>
@@ -7048,6 +8239,12 @@
         <f aca="false">IF($A197="","",IF($K197&lt;=0,"Rupture",IF($K197&lt;=N($H197),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N197" s="23"/>
+      <c r="O197" s="23"/>
+      <c r="P197" s="21" t="str">
+        <f aca="false">IF($A197="","",IF($K197&lt;=N($H197),MAX(0,2*N($H197)-$K197),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="23"/>
@@ -7078,6 +8275,12 @@
         <f aca="false">IF($A198="","",IF($K198&lt;=0,"Rupture",IF($K198&lt;=N($H198),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N198" s="23"/>
+      <c r="O198" s="23"/>
+      <c r="P198" s="21" t="str">
+        <f aca="false">IF($A198="","",IF($K198&lt;=N($H198),MAX(0,2*N($H198)-$K198),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="23"/>
@@ -7108,6 +8311,12 @@
         <f aca="false">IF($A199="","",IF($K199&lt;=0,"Rupture",IF($K199&lt;=N($H199),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N199" s="23"/>
+      <c r="O199" s="23"/>
+      <c r="P199" s="21" t="str">
+        <f aca="false">IF($A199="","",IF($K199&lt;=N($H199),MAX(0,2*N($H199)-$K199),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="23"/>
@@ -7138,6 +8347,12 @@
         <f aca="false">IF($A200="","",IF($K200&lt;=0,"Rupture",IF($K200&lt;=N($H200),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N200" s="23"/>
+      <c r="O200" s="23"/>
+      <c r="P200" s="21" t="str">
+        <f aca="false">IF($A200="","",IF($K200&lt;=N($H200),MAX(0,2*N($H200)-$K200),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="23"/>
@@ -7168,6 +8383,12 @@
         <f aca="false">IF($A201="","",IF($K201&lt;=0,"Rupture",IF($K201&lt;=N($H201),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N201" s="23"/>
+      <c r="O201" s="23"/>
+      <c r="P201" s="21" t="str">
+        <f aca="false">IF($A201="","",IF($K201&lt;=N($H201),MAX(0,2*N($H201)-$K201),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="23"/>
@@ -7198,6 +8419,12 @@
         <f aca="false">IF($A202="","",IF($K202&lt;=0,"Rupture",IF($K202&lt;=N($H202),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N202" s="23"/>
+      <c r="O202" s="23"/>
+      <c r="P202" s="21" t="str">
+        <f aca="false">IF($A202="","",IF($K202&lt;=N($H202),MAX(0,2*N($H202)-$K202),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="23"/>
@@ -7228,6 +8455,12 @@
         <f aca="false">IF($A203="","",IF($K203&lt;=0,"Rupture",IF($K203&lt;=N($H203),"À commander","OK")))</f>
         <v/>
       </c>
+      <c r="N203" s="23"/>
+      <c r="O203" s="23"/>
+      <c r="P203" s="21" t="str">
+        <f aca="false">IF($A203="","",IF($K203&lt;=N($H203),MAX(0,2*N($H203)-$K203),0))</f>
+        <v/>
+      </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="23"/>
@@ -7256,6 +8489,12 @@
       </c>
       <c r="M204" s="22" t="str">
         <f aca="false">IF($A204="","",IF($K204&lt;=0,"Rupture",IF($K204&lt;=N($H204),"À commander","OK")))</f>
+        <v/>
+      </c>
+      <c r="N204" s="23"/>
+      <c r="O204" s="23"/>
+      <c r="P204" s="21" t="str">
+        <f aca="false">IF($A204="","",IF($K204&lt;=N($H204),MAX(0,2*N($H204)-$K204),0))</f>
         <v/>
       </c>
     </row>
@@ -7307,56 +8546,56 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="25" t="n">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C5" s="26" t="str">
         <f aca="false">IF($B5="","",IFERROR(INDEX(Produits!$B$5:$B$204,MATCH($B5,Produits!$A$5:$A$204,0)),"Code inconnu"))</f>
         <v>EXEMPLE - Riz 25 kg</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="E5" s="20" t="n">
         <v>10</v>
@@ -7374,22 +8613,22 @@
         <v/>
       </c>
       <c r="I5" s="19" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="25" t="n">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C6" s="26" t="str">
         <f aca="false">IF($B6="","",IFERROR(INDEX(Produits!$B$5:$B$204,MATCH($B6,Produits!$A$5:$A$204,0)),"Code inconnu"))</f>
         <v>EXEMPLE - Riz 25 kg</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E6" s="20" t="n">
         <v>4</v>
@@ -7407,22 +8646,22 @@
         <v>120</v>
       </c>
       <c r="I6" s="19" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="25" t="n">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C7" s="26" t="str">
         <f aca="false">IF($B7="","",IFERROR(INDEX(Produits!$B$5:$B$204,MATCH($B7,Produits!$A$5:$A$204,0)),"Code inconnu"))</f>
         <v>EXEMPLE - Huile 5 L</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E7" s="20" t="n">
         <v>7</v>
@@ -7440,7 +8679,7 @@
         <v>84</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>